<commit_message>
added 20, 24, and 26 Tecan Files
</commit_message>
<xml_diff>
--- a/RAnalysis/data/Pacific_oyster/resazurin/20260630_28/NIFA_Resazurin_28_T0_30062026_1025_g77.xlsx
+++ b/RAnalysis/data/Pacific_oyster/resazurin/20260630_28/NIFA_Resazurin_28_T0_30062026_1025_g77.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\Documents\Tecan\SparkControl magellan\wsp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anna/Documents/Predictive_phenomics/RAnalysis/data/Pacific_oyster/resazurin/20260630_28/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0917088F-6ECD-45E9-9869-F1EA9A11E116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FEE3E76-EA03-F54B-9AAC-2A2FFEF19D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2556" yWindow="1212" windowWidth="17544" windowHeight="9732" xr2:uid="{EF07D611-BCD9-41A8-B33E-3AFBD801832F}"/>
+    <workbookView xWindow="2560" yWindow="1220" windowWidth="17540" windowHeight="9740" xr2:uid="{EF07D611-BCD9-41A8-B33E-3AFBD801832F}"/>
   </bookViews>
   <sheets>
     <sheet name="SparkControl magellan Sheet 1" sheetId="1" r:id="rId1"/>
@@ -162,7 +162,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -528,521 +528,521 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D8F1F14-B98C-4AD0-AD50-D4CFAEA6F6FC}">
-  <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <dimension ref="A1:M52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
+      <c r="B44">
         <v>1</v>
       </c>
-      <c r="C1">
+      <c r="C44">
         <v>2</v>
       </c>
-      <c r="D1">
+      <c r="D44">
         <v>3</v>
       </c>
-      <c r="E1">
+      <c r="E44">
         <v>4</v>
       </c>
-      <c r="F1">
+      <c r="F44">
         <v>5</v>
       </c>
-      <c r="G1">
+      <c r="G44">
         <v>6</v>
       </c>
-      <c r="H1">
+      <c r="H44">
         <v>7</v>
       </c>
-      <c r="I1">
+      <c r="I44">
         <v>8</v>
       </c>
-      <c r="J1">
-        <v>9</v>
-      </c>
-      <c r="K1">
+      <c r="J44">
+        <v>9</v>
+      </c>
+      <c r="K44">
         <v>10</v>
       </c>
-      <c r="L1">
+      <c r="L44">
         <v>11</v>
       </c>
-      <c r="M1">
+      <c r="M44">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B45">
         <v>2426</v>
       </c>
-      <c r="C2">
+      <c r="C45">
         <v>2516</v>
       </c>
-      <c r="D2">
+      <c r="D45">
         <v>2554</v>
       </c>
-      <c r="E2">
+      <c r="E45">
         <v>2383</v>
       </c>
-      <c r="F2">
+      <c r="F45">
         <v>2403</v>
       </c>
-      <c r="G2">
+      <c r="G45">
         <v>2612</v>
       </c>
-      <c r="H2">
+      <c r="H45">
         <v>2652</v>
       </c>
-      <c r="I2">
+      <c r="I45">
         <v>2513</v>
       </c>
-      <c r="J2">
+      <c r="J45">
         <v>2389</v>
       </c>
-      <c r="K2">
+      <c r="K45">
         <v>2754</v>
       </c>
-      <c r="L2">
+      <c r="L45">
         <v>2501</v>
       </c>
-      <c r="M2">
+      <c r="M45">
         <v>2540</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B46">
         <v>2492</v>
       </c>
-      <c r="C3">
+      <c r="C46">
         <v>2445</v>
       </c>
-      <c r="D3">
+      <c r="D46">
         <v>2650</v>
       </c>
-      <c r="E3">
+      <c r="E46">
         <v>2448</v>
       </c>
-      <c r="F3">
+      <c r="F46">
         <v>2810</v>
       </c>
-      <c r="G3">
+      <c r="G46">
         <v>2657</v>
       </c>
-      <c r="H3">
+      <c r="H46">
         <v>2507</v>
       </c>
-      <c r="I3">
+      <c r="I46">
         <v>2635</v>
       </c>
-      <c r="J3">
+      <c r="J46">
         <v>2490</v>
       </c>
-      <c r="K3">
+      <c r="K46">
         <v>2484</v>
       </c>
-      <c r="L3">
+      <c r="L46">
         <v>2484</v>
       </c>
-      <c r="M3">
+      <c r="M46">
         <v>2795</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B47">
         <v>2690</v>
       </c>
-      <c r="C4">
+      <c r="C47">
         <v>2562</v>
       </c>
-      <c r="D4">
+      <c r="D47">
         <v>2821</v>
       </c>
-      <c r="E4">
+      <c r="E47">
         <v>2649</v>
       </c>
-      <c r="F4">
+      <c r="F47">
         <v>2370</v>
       </c>
-      <c r="G4">
+      <c r="G47">
         <v>2840</v>
       </c>
-      <c r="H4">
+      <c r="H47">
         <v>2418</v>
       </c>
-      <c r="I4">
+      <c r="I47">
         <v>2343</v>
       </c>
-      <c r="J4">
+      <c r="J47">
         <v>2363</v>
       </c>
-      <c r="K4">
+      <c r="K47">
         <v>2893</v>
       </c>
-      <c r="L4">
+      <c r="L47">
         <v>2827</v>
       </c>
-      <c r="M4">
+      <c r="M47">
         <v>3038</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B48">
         <v>2938</v>
       </c>
-      <c r="C5">
+      <c r="C48">
         <v>2403</v>
       </c>
-      <c r="D5">
+      <c r="D48">
         <v>2726</v>
       </c>
-      <c r="E5">
+      <c r="E48">
         <v>2504</v>
       </c>
-      <c r="F5">
+      <c r="F48">
         <v>2602</v>
       </c>
-      <c r="G5">
+      <c r="G48">
         <v>2977</v>
       </c>
-      <c r="H5">
+      <c r="H48">
         <v>2495</v>
       </c>
-      <c r="I5">
+      <c r="I48">
         <v>2315</v>
       </c>
-      <c r="J5">
+      <c r="J48">
         <v>2524</v>
       </c>
-      <c r="K5">
+      <c r="K48">
         <v>2665</v>
       </c>
-      <c r="L5">
+      <c r="L48">
         <v>2903</v>
       </c>
-      <c r="M5">
+      <c r="M48">
         <v>2619</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B49">
         <v>2909</v>
       </c>
-      <c r="C6">
+      <c r="C49">
         <v>2729</v>
       </c>
-      <c r="D6">
+      <c r="D49">
         <v>2958</v>
       </c>
-      <c r="E6">
+      <c r="E49">
         <v>2632</v>
       </c>
-      <c r="F6">
+      <c r="F49">
         <v>2375</v>
       </c>
-      <c r="G6">
+      <c r="G49">
         <v>2642</v>
       </c>
-      <c r="H6">
+      <c r="H49">
         <v>2547</v>
       </c>
-      <c r="I6">
+      <c r="I49">
         <v>2300</v>
       </c>
-      <c r="J6">
+      <c r="J49">
         <v>2802</v>
       </c>
-      <c r="K6">
+      <c r="K49">
         <v>2459</v>
       </c>
-      <c r="L6">
+      <c r="L49">
         <v>2422</v>
       </c>
-      <c r="M6">
+      <c r="M49">
         <v>2706</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B50">
         <v>2497</v>
       </c>
-      <c r="C7">
+      <c r="C50">
         <v>2612</v>
       </c>
-      <c r="D7">
+      <c r="D50">
         <v>2543</v>
       </c>
-      <c r="E7">
+      <c r="E50">
         <v>2758</v>
       </c>
-      <c r="F7">
+      <c r="F50">
         <v>2430</v>
       </c>
-      <c r="G7">
+      <c r="G50">
         <v>2709</v>
       </c>
-      <c r="H7">
+      <c r="H50">
         <v>2391</v>
       </c>
-      <c r="I7">
+      <c r="I50">
         <v>2248</v>
       </c>
-      <c r="J7">
+      <c r="J50">
         <v>2428</v>
       </c>
-      <c r="K7">
+      <c r="K50">
         <v>2569</v>
       </c>
-      <c r="L7">
+      <c r="L50">
         <v>2510</v>
       </c>
-      <c r="M7">
+      <c r="M50">
         <v>2602</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="1" t="s">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B51">
         <v>2269</v>
       </c>
-      <c r="C8">
+      <c r="C51">
         <v>2368</v>
       </c>
-      <c r="D8">
+      <c r="D51">
         <v>2262</v>
       </c>
-      <c r="E8">
+      <c r="E51">
         <v>2489</v>
       </c>
-      <c r="F8">
+      <c r="F51">
         <v>2239</v>
       </c>
-      <c r="G8">
+      <c r="G51">
         <v>2450</v>
       </c>
-      <c r="H8">
+      <c r="H51">
         <v>2266</v>
       </c>
-      <c r="I8">
+      <c r="I51">
         <v>3100</v>
       </c>
-      <c r="J8">
+      <c r="J51">
         <v>2271</v>
       </c>
-      <c r="K8">
+      <c r="K51">
         <v>2646</v>
       </c>
-      <c r="L8">
+      <c r="L51">
         <v>2181</v>
       </c>
-      <c r="M8">
+      <c r="M51">
         <v>2678</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="1" t="s">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
-      <c r="A16" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1">
-      <c r="A26" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1">
-      <c r="A27" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1">
-      <c r="A28" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1">
-      <c r="A29" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1">
-      <c r="A30" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1">
-      <c r="A31" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1">
-      <c r="A32" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1">
-      <c r="A35" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1">
-      <c r="A36" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="1" t="s">
-        <v>38</v>
+      <c r="B52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>